<commit_message>
Extend general contractor run to 16 companies
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UDKoKe43tCUJkVykefgCLw
</commit_message>
<xml_diff>
--- a/gc_new_contacts.xlsx
+++ b/gc_new_contacts.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Needs Manual Research" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$E$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Manual Research'!$A$1:$D$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Manual Research'!$A$1:$D$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Renee Er***t</t>
+          <t>Renee Ernst</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1041,17 +1041,179 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>renee@legacymcs.com</t>
+          <t>renee@legacydcs.com</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Pattern-based - verify before sending</t>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>HITT Contracting</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Jennifer Macks</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Vice President and Business Unit Leader</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>jmacks@hitt-gc.com</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Rand Construction</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Ryan McGovern</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>rmcgovern@randcc.com</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Rand Construction</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Zachary Clardy</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Director of Field Operations</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>clardy@randcc.com</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Gordon Highlander</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Lee Sawyer</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Vice President Business Development</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>lsawyer@gordonhighlander.com</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Gordon Highlander</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Brian Jarrett</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Vice President of Business Development</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>bjarrett@gordonhighlander.com</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Andres Construction</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Tom Feather</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>VP</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>tom@andresconstruction.com</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1062,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1453,34 +1615,34 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Jennifer Ma***s</t>
+          <t>Colby Cerelejia</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Vice President and Business Unit Leader</t>
+          <t>Human Resources Business Partner</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>Apollo has no email on file for this person</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HITT Contracting</t>
+          <t>Rand Construction</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Colby Ce***a</t>
+          <t>Matt Da***h</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Human Resources Business Partner</t>
+          <t>Principal</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1492,17 +1654,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Rand Construction</t>
+          <t>Gordon Highlander</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ryan Mc***n</t>
+          <t>Pam Do***n</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Director</t>
+          <t>Vice President of Strategic Partner Relationships</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1514,17 +1676,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Rand Construction</t>
+          <t>Gordon Highlander</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Zachary Cl***y</t>
+          <t>Kyle Hu***t</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Director of Field Operations</t>
+          <t>Director of Operations</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1536,17 +1698,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Rand Construction</t>
+          <t>Gordon Highlander</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Matt Da***h</t>
+          <t>Stephanie Bo***l</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Principal</t>
+          <t>Associate Director of Preconstruction</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1563,12 +1725,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Lee Sa***r</t>
+          <t>Heidi Ma***e</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Vice President Business Development</t>
+          <t>Project Coordinator, Marketing Director</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1580,17 +1742,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Gordon Highlander</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Brian Ja***t</t>
+          <t>Caren Wi***h</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Vice President of Business Development</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1602,17 +1764,17 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Gordon Highlander</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Pam Do***n</t>
+          <t>Jennifer Fe***s</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Vice President of Strategic Partner Relationships</t>
+          <t>Marketing Manager</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1624,17 +1786,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Gordon Highlander</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Kyle Hu***t</t>
+          <t>Anson Wa***g</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Director of Operations</t>
+          <t>Director of Construction</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1646,17 +1808,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Gordon Highlander</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Stephanie Bo***l</t>
+          <t>Wade Ba***r</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Associate Director of Preconstruction</t>
+          <t>Director of Engineering</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1668,17 +1830,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Gordon Highlander</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Heidi Ma***e</t>
+          <t>Michael Jo***n</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Project Coordinator, Marketing Director</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1690,17 +1852,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Andres Construction</t>
+          <t>Headwater Construction</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Tom Fe***r</t>
+          <t>Logan Wa***s</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>VP</t>
+          <t>VP of Capital Relations</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1712,207 +1874,75 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Caren Wi***h</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Vice President</t>
-        </is>
-      </c>
+          <t>Burton Construction</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Jennifer Fe***s</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Marketing Manager</t>
-        </is>
-      </c>
+          <t>Weis Builders</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Anson Wa***g</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Director of Construction</t>
-        </is>
-      </c>
+          <t>Jay-Reese</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Wade Ba***r</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Director of Engineering</t>
-        </is>
-      </c>
+          <t>Paradigm Commercial</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Michael Jo***n</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
+          <t>G. Creek Construction</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Logan Wa***s</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>VP of Capital Relations</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Burton Construction</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
           <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Weis Builders</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Jay-Reese</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Paradigm Commercial</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr"/>
-      <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>G. Creek Construction</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D40"/>
+  <autoFilter ref="A1:D34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Pin companies by Apollo org id and finish the general contractor batch
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UDKoKe43tCUJkVykefgCLw
</commit_message>
<xml_diff>
--- a/gc_new_contacts.xlsx
+++ b/gc_new_contacts.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Needs Manual Research" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$E$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Manual Research'!$A$1:$D$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Manual Research'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1212,8 +1212,116 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Headwater Construction</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Caren Williams-Murch</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Vice President</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>caren@hw-companies.com</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Headwater Construction</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Jennifer Feikis</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Manager</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>jennifer@hw-companies.com</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Verified by Apollo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Headwater Construction</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Anson Wa***g</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Director of Construction</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>anson@hw-companies.com</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Pattern-based - verify before sending</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Headwater Construction</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Wade Ba***r</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Director of Engineering</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>wade@hw-companies.com</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Pattern-based - verify before sending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
+  <autoFilter ref="A1:E32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1224,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1742,207 +1850,75 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Caren Wi***h</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Vice President</t>
-        </is>
-      </c>
+          <t>Burton Construction</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Jennifer Fe***s</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Marketing Manager</t>
-        </is>
-      </c>
+          <t>Weis Builders</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Anson Wa***g</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Director of Construction</t>
-        </is>
-      </c>
+          <t>Jay-Reese</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Wade Ba***r</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Director of Engineering</t>
-        </is>
-      </c>
+          <t>Paradigm Commercial</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
+          <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Michael Jo***n</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
+          <t>G. Creek Construction</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Headwater Construction</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Logan Wa***s</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>VP of Capital Relations</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Surname masked by Apollo and this domain's format needs it</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Burton Construction</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
           <t>No matching people in Apollo for the Austin corridor</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Weis Builders</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr"/>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Jay-Reese</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Paradigm Commercial</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>G. Creek Construction</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>No matching people in Apollo for the Austin corridor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D34"/>
+  <autoFilter ref="A1:D28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>